<commit_message>
Refactor data loading and remove OKX caching script. Update main.py to eliminate OKX candle downloads and adjust README files accordingly. Enhance data files for BTC, ETH, and SOL with updated forecasts and predictions. Modify visualization files for improved clarity and interactivity.
</commit_message>
<xml_diff>
--- a/exports/btc-usd_forecast_next7.xlsx
+++ b/exports/btc-usd_forecast_next7.xlsx
@@ -443,71 +443,71 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025-11-15</t>
+          <t>2025-11-17</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>94092.49000000001</v>
+        <v>94786.66</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-11-16</t>
+          <t>2025-11-18</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>94109.49000000001</v>
+        <v>94901.73</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-11-17</t>
+          <t>2025-11-19</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>94704.02</v>
+        <v>95406.66</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2025-11-18</t>
+          <t>2025-11-20</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>94864.87</v>
+        <v>95776.16</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2025-11-19</t>
+          <t>2025-11-21</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>95273.05</v>
+        <v>95616.09</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2025-11-20</t>
+          <t>2025-11-22</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>95748.95</v>
+        <v>95539.67999999999</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2025-11-21</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>95687.57000000001</v>
+        <v>95249.42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove presentation outline and update README for clarity on project objectives. Update various data and export files, including BTC, ETH, and SOL forecasts and predictions, along with visualizations for improved interactivity.
</commit_message>
<xml_diff>
--- a/exports/btc-usd_forecast_next7.xlsx
+++ b/exports/btc-usd_forecast_next7.xlsx
@@ -443,71 +443,71 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025-11-17</t>
+          <t>2025-11-21</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>94786.66</v>
+        <v>86468.27</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-11-18</t>
+          <t>2025-11-22</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>94901.73</v>
+        <v>86579.46000000001</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-11-19</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>95406.66</v>
+        <v>86662.10000000001</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2025-11-20</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>95776.16</v>
+        <v>86184.2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2025-11-21</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>95616.09</v>
+        <v>86195.17</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>95539.67999999999</v>
+        <v>86374.49000000001</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>95249.42</v>
+        <v>86030.87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor main.py to implement rolling backtest for linear regression predictions, enhancing the prediction comparison function to include training dates. Update .gitignore to remove unnecessary entries and clean up documentation in various source files. Update data files for BTC, ETH, and SOL with new predictions and forecasts, along with corresponding visualizations for improved clarity.
</commit_message>
<xml_diff>
--- a/exports/btc-usd_forecast_next7.xlsx
+++ b/exports/btc-usd_forecast_next7.xlsx
@@ -443,71 +443,71 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025-11-21</t>
+          <t>2025-11-22</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>86468.27</v>
+        <v>85197.05</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>86579.46000000001</v>
+        <v>85240.13</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>86662.10000000001</v>
+        <v>84764.75999999999</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>86184.2</v>
+        <v>84676.09</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>86195.17</v>
+        <v>84877.37</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>86374.49000000001</v>
+        <v>84666.73</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>86030.87</v>
+        <v>84173.85000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>